<commit_message>
VRPA-00003: Finalized Code for Machine Transfer
</commit_message>
<xml_diff>
--- a/data/Processing-Report.xlsx
+++ b/data/Processing-Report.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="21029"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D6B5865-48FA-4E70-B748-71D8154225E2}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17C909E7-F762-402C-BB5B-839061752C08}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8868" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Date and time processing started</t>
   </si>
@@ -69,6 +69,12 @@
   </si>
   <si>
     <t>Count after Employment Date Filter</t>
+  </si>
+  <si>
+    <t>Count after Civil Labourer Roles</t>
+  </si>
+  <si>
+    <t>Count after Production Worker Role</t>
   </si>
 </sst>
 </file>
@@ -454,7 +460,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:T1"/>
   <sheetFormatPr defaultRowHeight="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.77734375" customWidth="1"/>
@@ -474,7 +480,7 @@
     <col min="15" max="15" width="8.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="1" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" s="1" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -528,6 +534,12 @@
       </c>
       <c r="R1" s="1" t="s">
         <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>